<commit_message>
Added SCP file access to tg_bot
</commit_message>
<xml_diff>
--- a/Attendence list.xlsx
+++ b/Attendence list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Personal\Wind3style\workspace\xc_export\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E4E5D61-AF0E-4E9C-8718-B599A59C6722}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F179662-F2AC-469B-A8E7-3F2B29762E05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{C5209F01-11F8-4536-83CC-330C0F186448}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
   <si>
     <t>Number</t>
   </si>
@@ -106,6 +106,9 @@
   </si>
   <si>
     <t>Veronika Blagoveshchenskaya</t>
+  </si>
+  <si>
+    <t>tg_username</t>
   </si>
 </sst>
 </file>
@@ -467,153 +470,159 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51BB7798-2C08-49E6-835C-257ED4D1D79F}">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.5546875" customWidth="1"/>
-    <col min="3" max="3" width="28.5546875" customWidth="1"/>
+    <col min="1" max="2" width="16.5546875" customWidth="1"/>
+    <col min="4" max="4" width="28.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="2"/>
+      <c r="C2" s="2">
         <v>1</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="2"/>
+      <c r="C3" s="2">
         <v>2</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4" s="2"/>
+      <c r="C4" s="2">
         <v>3</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B5" t="s">
         <v>3</v>
       </c>
-      <c r="B5">
+      <c r="C5">
         <v>4</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>6</v>
       </c>
-      <c r="B6">
+      <c r="C6">
         <v>5</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>8</v>
       </c>
-      <c r="B7">
+      <c r="C7">
         <v>6</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>12</v>
       </c>
-      <c r="B8">
+      <c r="C8">
         <v>7</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>13</v>
       </c>
-      <c r="B9">
+      <c r="C9">
         <v>8</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>15</v>
       </c>
-      <c r="B10">
+      <c r="C10">
         <v>9</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>18</v>
       </c>
-      <c r="B11">
+      <c r="C11">
         <v>10</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>19</v>
       </c>
-      <c r="B12">
+      <c r="C12">
         <v>11</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>21</v>
       </c>
-      <c r="B13">
+      <c r="C13">
         <v>12</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>22</v>
       </c>
     </row>

</xml_diff>